<commit_message>
refactor: preserve trophy humor/flavor with blended parenthetical
preserve trophy humor/flavor with blended parenthetical mechanical
requirements
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/trophies.xlsx
+++ b/mod_project/data_tables/trophies.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Defeat your first dark mutant in the main story.</t>
+          <t>Defeated your first dark mutant.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Assemble a party member of each base class (5 classes).</t>
+          <t>Assembled a party member of each base class. (5 classes)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Recruit 9 members of the Royal Library squad.</t>
+          <t>Reassembled half of the old Royal Library squad. (9 members)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Recruit 10 heroine party members.</t>
+          <t>Assembled a healthy number of party members. (10 heroines)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Recruit all 18 members of the Royal Library squad.</t>
+          <t>Reassembled the entire old Royal Library squad. (18 heroines)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Win 300 battles.</t>
+          <t>Won 300 battles.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Win 600 battles.</t>
+          <t>Won 600 battles.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Win 1,200 battles.</t>
+          <t>Won 1,200 battles.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Win 2,000 battles.</t>
+          <t>Won 2,000 battles.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Create 75 sealbooks at the Seal Control Room.</t>
+          <t>Created 75 sealbooks.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Create 150 sealbooks at the Seal Control Room.</t>
+          <t>Created 150 sealbooks.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Create 225 sealbooks at the Seal Control Room.</t>
+          <t>Created 225 sealbooks.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Create 300 sealbooks at the Seal Control Room.</t>
+          <t>Created 300 sealbooks.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Create all 22 Grand Sealbooks from dark mutants.</t>
+          <t>Created every grand sealbook. (22 mutant seals)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>View 50 sub events across base facilities.</t>
+          <t>Saw 50 or more sub events.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>View 100 sub events across base facilities.</t>
+          <t>Saw 100 or more sub events.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>View 200 sub events across base facilities.</t>
+          <t>Saw 200 or more sub events.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Advance all 18 heroines to an intermediate class (Lv15+).</t>
+          <t>Reached an intermediate class with everyone. (All 18 at Lv 15+)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Advance all 18 heroines to an advanced class (Lv30+).</t>
+          <t>Reached an advanced class with everyone. (All 18 at Lv 30+)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Unlock and change to all 32 classes across the roster.</t>
+          <t>Changed to all possible classes. (Unlock all 32 classes)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Learn all skills across all classes on any heroine.</t>
+          <t>Learned all skills. (Master all class skills on one heroine)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Form all 20 unique party skill compositions.</t>
+          <t>Activated all party skills. (Trigger all 20 party compositions)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Execute 26 different joint skills in battle.</t>
+          <t>Activated half of all joint skills. (Execute 26 joint skills)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Execute all 52 unique joint skills in battle.</t>
+          <t>Activated all joint skills. (Execute all 52 joint skills)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Purchase and consume all 16 Ramen and Ice Cream meals.</t>
+          <t>Sampled every flavor of Ramen and Ice Cream. (Eat all 16 meals)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Encounter the wandering dungeon peddler 30 times.</t>
+          <t>Encountered the peddler many, many times. (30 encounters)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Forge equipment at Black Mary's smithy 100 times.</t>
+          <t>Enchanted equipment more than 100 times.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Unlock class outfits for all 18 heroines.</t>
+          <t>Purchased class outfits for the entire team. (18 heroines)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hire tavern mercenaries 30 times.</t>
+          <t>Hired the services of mercenaries many times. (30 hires)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Reach maximum Client Rank 20 at the Quest Desk.</t>
+          <t>Maxed out client level at the Quest Desk. (Rank 20)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Defeat instructor Irena in the tavern challenge match.</t>
+          <t>Tempted your instructor to test your power. (Defeat Irena)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Defeat the three Magi heroes in the post-game dungeon.</t>
+          <t>Defeated a certain trio of historical heroes. (Beat the Magi)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Defeat all Therian beastkin monster variants.</t>
+          <t>Defeated every type of Therian enemy. (All Therian variants)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Defeat the 4 wandering aimless warrior bosses.</t>
+          <t>Ended the wanderings of four aimless warriors. (Defeat 4 wanderers)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pay off Lolo's 10,000 gold debt in full.</t>
+          <t>Paid off Lolo's loan for her. (Repay 10,000 gold debt)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Open 300 treasure chests across all dungeons.</t>
+          <t>Opened an absurd number of chests. (Open 300 chests)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Accumulate over 777,777 gold in party funds.</t>
+          <t>Amassed over 777,777 gold.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Successfully escape from 100 dungeon battles.</t>
+          <t>Lived to fight another day... a lot. (Escape 100 battles)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Transform 100 monsters into items with Materialize.</t>
+          <t>Snackified every monster with Materialize. (100 item drops)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fully explore and map 50% of all dungeon floors.</t>
+          <t>Mapped half of all dungeon floors. (50% map completion)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fully explore and map 90% of all dungeon floors.</t>
+          <t>Mapped almost all dungeon floors. (90% map completion)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Trigger 100 dungeon floor traps.</t>
+          <t>Got caught in a painful number of traps. (Trigger 100 traps)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Attain Crown status (Level 99 + Level Reset) on any heroine.</t>
+          <t>Attained a crown. (Reach Lv 99 and perform Level Reset)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Defeat 50 enemies using autonomous Sealbook Summons.</t>
+          <t>Let a Sealbook Summon finish off many foes. (50 summon kills)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Raise any heroine to maximum Level 99.</t>
+          <t>Transcended humanity to seize the godhead. (Reach Level 99)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Defeat the ancient dragon superboss in the EX dungeon.</t>
+          <t>Trounced the rampaging wicked dragon. (Defeat ancient dragon)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Defeat casino owner boss Gous-shin in the post-game.</t>
+          <t>Trounced the miserly casino owner. (Defeat Gous-shin)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Defeat Queen Elizabeth in the post-game EX dungeon.</t>
+          <t>Trounced the inappropriate queen. Propriety! (Beat Elizabeth)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Defeat the Creator God superboss in the ultimate dungeon.</t>
+          <t>Trounced God? JRPG Complete? (Defeat Creator God)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Complete all post-game depths and clear the game.</t>
+          <t>Reached the end of the path to power. (Clear all EX depths)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">

</xml_diff>